<commit_message>
feat(question-bank): add dynamic demo excel generator and downloadable demo sheet in question modals
</commit_message>
<xml_diff>
--- a/public/templates/Skillizee_Grade6_Math_Questions_Demo.xlsx
+++ b/public/templates/Skillizee_Grade6_Math_Questions_Demo.xlsx
@@ -5,8 +5,7 @@
   <sheets>
     <sheet name="Questions" sheetId="1" r:id="rId1"/>
     <sheet name="Instructions" sheetId="2" r:id="rId2"/>
-    <sheet name="Examples" sheetId="3" r:id="rId3"/>
-    <sheet name="Activity List" sheetId="4" r:id="rId4"/>
+    <sheet name="Activity List" sheetId="3" r:id="rId3"/>
   </sheets>
 </workbook>
 </file>
@@ -400,584 +399,979 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K16"/>
+  <dimension ref="A1:K30"/>
   <cols>
-    <col min="1" max="1" width="30.83203125" customWidth="1"/>
-    <col min="2" max="2" width="32.83203125" customWidth="1"/>
+    <col min="1" max="1" width="28.83203125" customWidth="1"/>
+    <col min="2" max="2" width="28.83203125" customWidth="1"/>
     <col min="3" max="3" width="65.83203125" customWidth="1"/>
-    <col min="4" max="4" width="22.83203125" customWidth="1"/>
-    <col min="5" max="5" width="22.83203125" customWidth="1"/>
-    <col min="6" max="6" width="22.83203125" customWidth="1"/>
-    <col min="7" max="7" width="22.83203125" customWidth="1"/>
+    <col min="4" max="4" width="20.83203125" customWidth="1"/>
+    <col min="5" max="5" width="20.83203125" customWidth="1"/>
+    <col min="6" max="6" width="20.83203125" customWidth="1"/>
+    <col min="7" max="7" width="20.83203125" customWidth="1"/>
     <col min="8" max="8" width="16.83203125" customWidth="1"/>
-    <col min="9" max="9" width="50.83203125" customWidth="1"/>
+    <col min="9" max="9" width="55.83203125" customWidth="1"/>
     <col min="10" max="10" width="14.83203125" customWidth="1"/>
-    <col min="11" max="11" width="32.83203125" customWidth="1"/>
+    <col min="11" max="11" width="30.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Activity</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Topic</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Question</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Option A</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Option B</v>
-      </c>
-      <c r="F1" t="str">
-        <v>Option C</v>
-      </c>
-      <c r="G1" t="str">
-        <v>Option D</v>
-      </c>
-      <c r="H1" t="str">
-        <v>Correct Answer</v>
-      </c>
-      <c r="I1" t="str">
-        <v>Explanation</v>
-      </c>
-      <c r="J1" t="str">
-        <v>Difficulty</v>
-      </c>
-      <c r="K1" t="str">
-        <v>Tags</v>
+        <v>SKILLIZEE ARCADE — GRADE 6 DEMO QUESTIONS DATASET</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Graphworks</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Data Handling &amp; Graphs</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Which ordered pair represents 3 units right on the x-axis and 4 units up on the y-axis?</v>
-      </c>
-      <c r="D2" t="str">
-        <v>(4, 3)</v>
-      </c>
-      <c r="E2" t="str">
-        <v>(3, 4)</v>
-      </c>
-      <c r="F2" t="str">
-        <v>(3, 0)</v>
-      </c>
-      <c r="G2" t="str">
-        <v>(0, 4)</v>
-      </c>
-      <c r="H2" t="str">
-        <v>B</v>
-      </c>
-      <c r="I2" t="str">
-        <v>Coordinates are written as (x, y). Moving 3 units right gives x = 3, and 4 units up gives y = 4, resulting in (3, 4).</v>
-      </c>
-      <c r="J2" t="str">
-        <v>Easy</v>
-      </c>
-      <c r="K2" t="str">
-        <v>Coordinates, Grid, Plotting</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>The Chocolate Factory</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Fractions</v>
-      </c>
-      <c r="C3" t="str">
-        <v>A chocolate batch uses 3/4 cup of melted cocoa. How much cocoa is needed for 3 full batches?</v>
-      </c>
-      <c r="D3" t="str">
-        <v>2 1/4 cups</v>
-      </c>
-      <c r="E3" t="str">
-        <v>1 1/2 cups</v>
-      </c>
-      <c r="F3" t="str">
-        <v>3 cups</v>
-      </c>
-      <c r="G3" t="str">
-        <v>9/4 cups</v>
-      </c>
-      <c r="H3" t="str">
-        <v>A</v>
-      </c>
-      <c r="I3" t="str">
-        <v>3 × 3/4 = 9/4 = 2 1/4 cups of cocoa.</v>
-      </c>
-      <c r="J3" t="str">
-        <v>Medium</v>
-      </c>
-      <c r="K3" t="str">
-        <v>Fractions, Multiplication, Mixed Numbers</v>
+        <v>This demo sheet contains pre-filled questions across all 13 arcade activities for testing and direct import into Skillizee Arcade.</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Percentage Harvest</v>
+        <v>Activity</v>
       </c>
       <c r="B4" t="str">
-        <v>Percentages</v>
+        <v>Topic</v>
       </c>
       <c r="C4" t="str">
-        <v>What is 20% of 80 kg of harvest apples?</v>
+        <v>Question</v>
       </c>
       <c r="D4" t="str">
-        <v>12 kg</v>
+        <v>Option A</v>
       </c>
       <c r="E4" t="str">
-        <v>16 kg</v>
+        <v>Option B</v>
       </c>
       <c r="F4" t="str">
-        <v>18 kg</v>
+        <v>Option C</v>
       </c>
       <c r="G4" t="str">
-        <v>20 kg</v>
+        <v>Option D</v>
       </c>
       <c r="H4" t="str">
-        <v>B</v>
+        <v>Correct Answer</v>
       </c>
       <c r="I4" t="str">
-        <v>20% of 80 = 0.2 × 80 = 16 kg.</v>
+        <v>Explanation</v>
       </c>
       <c r="J4" t="str">
-        <v>Easy</v>
+        <v>Difficulty</v>
       </c>
       <c r="K4" t="str">
-        <v>Percentages, Harvest, Calculations</v>
+        <v>Tags</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Park Planner</v>
+        <v>Math Escape Vault</v>
       </c>
       <c r="B5" t="str">
-        <v>Position &amp; Transformation</v>
+        <v>Place Value &amp; Decimals</v>
       </c>
       <c r="C5" t="str">
-        <v>When the point (2, 5) is reflected over the y-axis, what are its new coordinates?</v>
+        <v>In the number 542,891, what is the place value of the digit 4?</v>
       </c>
       <c r="D5" t="str">
-        <v>(-2, 5)</v>
+        <v>400</v>
       </c>
       <c r="E5" t="str">
-        <v>(2, -5)</v>
+        <v>4,000</v>
       </c>
       <c r="F5" t="str">
-        <v>(-2, -5)</v>
+        <v>40,000</v>
       </c>
       <c r="G5" t="str">
-        <v>(5, 2)</v>
+        <v>400,000</v>
       </c>
       <c r="H5" t="str">
-        <v>A</v>
+        <v>C</v>
       </c>
       <c r="I5" t="str">
-        <v>Reflecting over the y-axis negates the x-coordinate while y remains unchanged: (-2, 5).</v>
+        <v>The digit 4 is in the ten thousands place, so its value is 40,000.</v>
       </c>
       <c r="J5" t="str">
-        <v>Medium</v>
+        <v>Easy</v>
       </c>
       <c r="K5" t="str">
-        <v>Transformations, Reflection, Coordinates</v>
+        <v>Place Value, Decimals, Vault</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Ratio Rush</v>
+        <v>Math Escape Vault</v>
       </c>
       <c r="B6" t="str">
-        <v>Ratios, Rates &amp; Proportions</v>
+        <v>Place Value &amp; Decimals</v>
       </c>
       <c r="C6" t="str">
-        <v>A film studio uses 2 cameras for every 3 actors. If there are 12 actors, how many cameras are needed?</v>
+        <v>Evaluate the vault security pin code: 0.6 × 0.08</v>
       </c>
       <c r="D6" t="str">
-        <v>6</v>
+        <v>0.48</v>
       </c>
       <c r="E6" t="str">
-        <v>8</v>
+        <v>0.048</v>
       </c>
       <c r="F6" t="str">
-        <v>9</v>
+        <v>0.0048</v>
       </c>
       <c r="G6" t="str">
-        <v>10</v>
+        <v>4.8</v>
       </c>
       <c r="H6" t="str">
         <v>B</v>
       </c>
       <c r="I6" t="str">
-        <v>Scale factor is 12 ÷ 3 = 4. Cameras = 2 × 4 = 8.</v>
+        <v>6 × 8 = 48. With 1 + 2 = 3 decimal places, the answer is 0.048.</v>
       </c>
       <c r="J6" t="str">
-        <v>Easy</v>
+        <v>Medium</v>
       </c>
       <c r="K6" t="str">
-        <v>Ratio, Scaling, Unit Rate</v>
+        <v>Decimals, Multiplication</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Math Escape Vault</v>
+        <v>The Chocolate Factory</v>
       </c>
       <c r="B7" t="str">
-        <v>Place Value &amp; Decimals</v>
+        <v>Fractions</v>
       </c>
       <c r="C7" t="str">
-        <v>In the number 458.293, what is the place value of the digit 9?</v>
+        <v>A master chocolatier uses 3/4 kg of cocoa for one batch. How much cocoa is needed for 4 batches?</v>
       </c>
       <c r="D7" t="str">
-        <v>Tenths</v>
+        <v>2 kg</v>
       </c>
       <c r="E7" t="str">
-        <v>Hundredths</v>
+        <v>2 1/2 kg</v>
       </c>
       <c r="F7" t="str">
-        <v>Thousandths</v>
+        <v>3 kg</v>
       </c>
       <c r="G7" t="str">
-        <v>Tens</v>
+        <v>3 1/4 kg</v>
       </c>
       <c r="H7" t="str">
-        <v>B</v>
+        <v>C</v>
       </c>
       <c r="I7" t="str">
-        <v>The first digit after decimal is tenths (2), the second digit is hundredths (9).</v>
+        <v>4 × 3/4 = 12/4 = 3 kg.</v>
       </c>
       <c r="J7" t="str">
         <v>Easy</v>
       </c>
       <c r="K7" t="str">
-        <v>Place Value, Decimals</v>
+        <v>Fractions, Multiplication, Chocolate</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>The Great Number Railway</v>
+        <v>The Chocolate Factory</v>
       </c>
       <c r="B8" t="str">
-        <v>Operations &amp; Rounding</v>
+        <v>Fractions</v>
       </c>
       <c r="C8" t="str">
-        <v>Round 48,672 to the nearest thousand.</v>
+        <v>Simplify the fraction ratio of caramel fudge: 18/24</v>
       </c>
       <c r="D8" t="str">
-        <v>48,000</v>
+        <v>2/3</v>
       </c>
       <c r="E8" t="str">
-        <v>48,700</v>
+        <v>3/4</v>
       </c>
       <c r="F8" t="str">
-        <v>49,000</v>
+        <v>5/6</v>
       </c>
       <c r="G8" t="str">
-        <v>50,000</v>
+        <v>7/8</v>
       </c>
       <c r="H8" t="str">
-        <v>C</v>
+        <v>B</v>
       </c>
       <c r="I8" t="str">
-        <v>The hundreds digit is 6 (&gt;= 5), so we round up to 49,000.</v>
+        <v>Dividing numerator and denominator by GCD (6) gives 3/4.</v>
       </c>
       <c r="J8" t="str">
         <v>Easy</v>
       </c>
       <c r="K8" t="str">
-        <v>Rounding, Operations</v>
+        <v>Fractions, Simplification</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Carnival of Chance</v>
+        <v>Ratio Rush</v>
       </c>
       <c r="B9" t="str">
-        <v>Probability</v>
+        <v>Ratios, Rates &amp; Proportions</v>
       </c>
       <c r="C9" t="str">
-        <v>A carnival spinner has 8 equal sections numbered 1 to 8. What is the probability of landing on a prime number?</v>
+        <v>A film crew has 3 lighting rigs for every 5 cameras. If there are 25 cameras, how many lighting rigs are on set?</v>
       </c>
       <c r="D9" t="str">
-        <v>1/4</v>
+        <v>10</v>
       </c>
       <c r="E9" t="str">
-        <v>3/8</v>
+        <v>12</v>
       </c>
       <c r="F9" t="str">
-        <v>1/2</v>
+        <v>15</v>
       </c>
       <c r="G9" t="str">
-        <v>5/8</v>
+        <v>18</v>
       </c>
       <c r="H9" t="str">
         <v>C</v>
       </c>
       <c r="I9" t="str">
-        <v>The prime numbers between 1 and 8 are 2, 3, 5, 7 (4 numbers). Probability = 4/8 = 1/2.</v>
+        <v>Scale factor = 25 ÷ 5 = 5. Rigs = 3 × 5 = 15.</v>
       </c>
       <c r="J9" t="str">
-        <v>Medium</v>
+        <v>Easy</v>
       </c>
       <c r="K9" t="str">
-        <v>Probability, Primes, Spinner</v>
+        <v>Ratio, Scaling, Film Studio</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Blueprint Blitz</v>
+        <v>Ratio Rush</v>
       </c>
       <c r="B10" t="str">
-        <v>Shapes, Area &amp; Volume</v>
+        <v>Ratios, Rates &amp; Proportions</v>
       </c>
       <c r="C10" t="str">
-        <v>A rectangular prism has a length of 6 cm, width of 4 cm, and height of 5 cm. What is its volume?</v>
+        <v>A soundstage boom mic records 180 audio frames in 3 seconds. What is the recording rate per second?</v>
       </c>
       <c r="D10" t="str">
-        <v>60 cm³</v>
+        <v>45 frames/s</v>
       </c>
       <c r="E10" t="str">
-        <v>120 cm³</v>
+        <v>50 frames/s</v>
       </c>
       <c r="F10" t="str">
-        <v>148 cm³</v>
+        <v>60 frames/s</v>
       </c>
       <c r="G10" t="str">
-        <v>150 cm³</v>
+        <v>90 frames/s</v>
       </c>
       <c r="H10" t="str">
-        <v>B</v>
+        <v>C</v>
       </c>
       <c r="I10" t="str">
-        <v>Volume = length × width × height = 6 × 4 × 5 = 120 cm³.</v>
+        <v>Unit rate = 180 ÷ 3 = 60 frames per second.</v>
       </c>
       <c r="J10" t="str">
-        <v>Medium</v>
+        <v>Easy</v>
       </c>
       <c r="K10" t="str">
-        <v>Volume, 3D Shapes, Geometry</v>
+        <v>Unit Rate, Speed, Audio</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Equation Mission Control</v>
+        <v>Shape Shifter Arena</v>
       </c>
       <c r="B11" t="str">
-        <v>Expressions &amp; Equations</v>
+        <v>Geometry &amp; Symmetry</v>
       </c>
       <c r="C11" t="str">
-        <v>Solve for x: 3x + 7 = 22</v>
+        <v>What is the area of a neon battle arena rectangle with length 14 m and width 6 m?</v>
       </c>
       <c r="D11" t="str">
-        <v>x = 4</v>
+        <v>72 m²</v>
       </c>
       <c r="E11" t="str">
-        <v>x = 5</v>
+        <v>80 m²</v>
       </c>
       <c r="F11" t="str">
-        <v>x = 6</v>
+        <v>84 m²</v>
       </c>
       <c r="G11" t="str">
-        <v>x = 7</v>
+        <v>96 m²</v>
       </c>
       <c r="H11" t="str">
-        <v>B</v>
+        <v>C</v>
       </c>
       <c r="I11" t="str">
-        <v>Subtract 7 from both sides: 3x = 15. Divide by 3: x = 5.</v>
+        <v>Area = length × width = 14 × 6 = 84 m².</v>
       </c>
       <c r="J11" t="str">
-        <v>Medium</v>
+        <v>Easy</v>
       </c>
       <c r="K11" t="str">
-        <v>Algebra, Linear Equations</v>
+        <v>Area, Geometry, Rectangle</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Pattern Racers</v>
+        <v>Shape Shifter Arena</v>
       </c>
       <c r="B12" t="str">
-        <v>Sequences &amp; Functions</v>
+        <v>Geometry &amp; Symmetry</v>
       </c>
       <c r="C12" t="str">
-        <v>What is the 10th term in the sequence: 4, 7, 10, 13, ... ?</v>
+        <v>How many lines of symmetry does a regular hexagon shield possess?</v>
       </c>
       <c r="D12" t="str">
-        <v>28</v>
+        <v>3</v>
       </c>
       <c r="E12" t="str">
-        <v>31</v>
+        <v>4</v>
       </c>
       <c r="F12" t="str">
-        <v>34</v>
+        <v>5</v>
       </c>
       <c r="G12" t="str">
-        <v>37</v>
+        <v>6</v>
       </c>
       <c r="H12" t="str">
-        <v>B</v>
+        <v>D</v>
       </c>
       <c r="I12" t="str">
-        <v>The rule is 3n + 1. For n = 10, 3(10) + 1 = 31.</v>
+        <v>A regular polygon with n sides has n lines of symmetry. For a hexagon, n = 6.</v>
       </c>
       <c r="J12" t="str">
         <v>Medium</v>
       </c>
       <c r="K12" t="str">
-        <v>Sequences, nth term, Patterns</v>
+        <v>Symmetry, Polygons, Hexagon</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Decimal Delivery Network</v>
+        <v>Time Warp Train</v>
       </c>
       <c r="B13" t="str">
-        <v>Decimals</v>
+        <v>Time &amp; Measurement</v>
       </c>
       <c r="C13" t="str">
-        <v>Calculate: 14.75 × 0.4</v>
+        <v>The express steam train departs at 08:45 and reaches the next station at 11:15. How long was the journey?</v>
       </c>
       <c r="D13" t="str">
-        <v>5.8</v>
+        <v>2 hours 15 mins</v>
       </c>
       <c r="E13" t="str">
-        <v>5.9</v>
+        <v>2 hours 30 mins</v>
       </c>
       <c r="F13" t="str">
-        <v>6.1</v>
+        <v>2 hours 45 mins</v>
       </c>
       <c r="G13" t="str">
-        <v>59.0</v>
+        <v>3 hours</v>
       </c>
       <c r="H13" t="str">
         <v>B</v>
       </c>
       <c r="I13" t="str">
-        <v>14.75 × 0.4 = 5.9.</v>
+        <v>From 08:45 to 11:15 is 2 hours and 30 minutes.</v>
       </c>
       <c r="J13" t="str">
-        <v>Medium</v>
+        <v>Easy</v>
       </c>
       <c r="K13" t="str">
-        <v>Decimals, Multiplication</v>
+        <v>Elapsed Time, Clock, Train</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>The Solar Forge</v>
+        <v>Time Warp Train</v>
       </c>
       <c r="B14" t="str">
-        <v>Angles, Protractor &amp; Constructions</v>
+        <v>Time &amp; Measurement</v>
       </c>
       <c r="C14" t="str">
-        <v>Two angles are complementary. If one angle measures 38°, what is the measure of the second angle?</v>
+        <v>Convert 4.5 kilometers of railway track into meters.</v>
       </c>
       <c r="D14" t="str">
-        <v>42°</v>
+        <v>450 m</v>
       </c>
       <c r="E14" t="str">
-        <v>52°</v>
+        <v>4,050 m</v>
       </c>
       <c r="F14" t="str">
-        <v>62°</v>
+        <v>4,500 m</v>
       </c>
       <c r="G14" t="str">
-        <v>142°</v>
+        <v>45,000 m</v>
       </c>
       <c r="H14" t="str">
-        <v>B</v>
+        <v>C</v>
       </c>
       <c r="I14" t="str">
-        <v>Complementary angles add up to 90°. 90° - 38° = 52°.</v>
+        <v>1 km = 1,000 m. 4.5 × 1,000 = 4,500 m.</v>
       </c>
       <c r="J14" t="str">
         <v>Easy</v>
       </c>
       <c r="K14" t="str">
-        <v>Angles, Complementary, Geometry</v>
+        <v>Metric Conversion, Distance</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>The Chocolate Factory</v>
+        <v>Formula 1 Speedway</v>
       </c>
       <c r="B15" t="str">
-        <v>Fractions</v>
+        <v>Algebra &amp; Sequences</v>
       </c>
       <c r="C15" t="str">
-        <v>What is 5/6 ÷ 2/3 in simplest form?</v>
+        <v>Solve for the race car turbo boost level: 3x + 7 = 28</v>
       </c>
       <c r="D15" t="str">
-        <v>1 1/4</v>
+        <v>x = 5</v>
       </c>
       <c r="E15" t="str">
-        <v>5/9</v>
+        <v>x = 6</v>
       </c>
       <c r="F15" t="str">
-        <v>1 1/2</v>
+        <v>x = 7</v>
       </c>
       <c r="G15" t="str">
-        <v>10/18</v>
+        <v>x = 8</v>
       </c>
       <c r="H15" t="str">
-        <v>A</v>
+        <v>C</v>
       </c>
       <c r="I15" t="str">
-        <v>5/6 ÷ 2/3 = 5/6 × 3/2 = 15/12 = 5/4 = 1 1/4.</v>
+        <v>3x = 28 - 7 = 21, therefore x = 21 ÷ 3 = 7.</v>
       </c>
       <c r="J15" t="str">
-        <v>Hard</v>
+        <v>Medium</v>
       </c>
       <c r="K15" t="str">
-        <v>Fractions, Division, Mixed Numbers</v>
+        <v>Linear Equations, Algebra, Racing</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Ratio Rush</v>
+        <v>Formula 1 Speedway</v>
       </c>
       <c r="B16" t="str">
-        <v>Ratios, Rates &amp; Proportions</v>
+        <v>Algebra &amp; Sequences</v>
       </c>
       <c r="C16" t="str">
-        <v>A recipe uses 3 cups of flour to 2 cups of sugar. To make a larger batch using 15 cups of flour, how much sugar is needed?</v>
+        <v>Find the next term in the pit stop speed pattern: 4, 9, 14, 19, ___</v>
       </c>
       <c r="D16" t="str">
-        <v>8 cups</v>
+        <v>23</v>
       </c>
       <c r="E16" t="str">
-        <v>10 cups</v>
+        <v>24</v>
       </c>
       <c r="F16" t="str">
-        <v>12 cups</v>
+        <v>25</v>
       </c>
       <c r="G16" t="str">
-        <v>14 cups</v>
+        <v>26</v>
       </c>
       <c r="H16" t="str">
         <v>B</v>
       </c>
       <c r="I16" t="str">
-        <v>15 ÷ 3 = 5 (scaling factor). Sugar = 2 × 5 = 10 cups.</v>
+        <v>The sequence increases by +5 each step: 19 + 5 = 24.</v>
       </c>
       <c r="J16" t="str">
         <v>Easy</v>
       </c>
       <c r="K16" t="str">
-        <v>Ratio, Proportions, Scaling</v>
+        <v>Number Sequences, Patterns</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>Deep Sea Diver</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Integers &amp; Negative Numbers</v>
+      </c>
+      <c r="C17" t="str">
+        <v>A submarine dives from -45 meters down to -120 meters. What is the change in submarine depth?</v>
+      </c>
+      <c r="D17" t="str">
+        <v>-165 m</v>
+      </c>
+      <c r="E17" t="str">
+        <v>-75 m</v>
+      </c>
+      <c r="F17" t="str">
+        <v>+75 m</v>
+      </c>
+      <c r="G17" t="str">
+        <v>+165 m</v>
+      </c>
+      <c r="H17" t="str">
+        <v>B</v>
+      </c>
+      <c r="I17" t="str">
+        <v>Change = -120 - (-45) = -120 + 45 = -75 meters.</v>
+      </c>
+      <c r="J17" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="K17" t="str">
+        <v>Integers, Subtraction, Submarine</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>Deep Sea Diver</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Integers &amp; Negative Numbers</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Calculate the submarine cabin pressure differential: (-15) + (-28)</v>
+      </c>
+      <c r="D18" t="str">
+        <v>-13</v>
+      </c>
+      <c r="E18" t="str">
+        <v>-43</v>
+      </c>
+      <c r="F18" t="str">
+        <v>13</v>
+      </c>
+      <c r="G18" t="str">
+        <v>43</v>
+      </c>
+      <c r="H18" t="str">
+        <v>B</v>
+      </c>
+      <c r="I18" t="str">
+        <v>Adding two negatives: -15 + -28 = -43.</v>
+      </c>
+      <c r="J18" t="str">
+        <v>Easy</v>
+      </c>
+      <c r="K18" t="str">
+        <v>Negative Numbers, Addition</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>Percentage Harvest</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Percentages</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Out of 250 freshly harvested golden apples, 20% are packed for VIP delivery. How many apples is that?</v>
+      </c>
+      <c r="D19" t="str">
+        <v>40</v>
+      </c>
+      <c r="E19" t="str">
+        <v>45</v>
+      </c>
+      <c r="F19" t="str">
+        <v>50</v>
+      </c>
+      <c r="G19" t="str">
+        <v>60</v>
+      </c>
+      <c r="H19" t="str">
+        <v>C</v>
+      </c>
+      <c r="I19" t="str">
+        <v>20% of 250 = 0.20 × 250 = 50 apples.</v>
+      </c>
+      <c r="J19" t="str">
+        <v>Easy</v>
+      </c>
+      <c r="K19" t="str">
+        <v>Percentages, Harvest, Apples</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>Percentage Harvest</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Percentages</v>
+      </c>
+      <c r="C20" t="str">
+        <v>A farm basket price of  is discounted by 15%. What is the new sale price?</v>
+      </c>
+      <c r="D20" t="str">
+        <v/>
+      </c>
+      <c r="E20" t="str">
+        <v/>
+      </c>
+      <c r="F20" t="str">
+        <v/>
+      </c>
+      <c r="G20" t="str">
+        <v/>
+      </c>
+      <c r="H20" t="str">
+        <v>B</v>
+      </c>
+      <c r="I20" t="str">
+        <v>Discount = 15% of  = . New price =  -  = .</v>
+      </c>
+      <c r="J20" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="K20" t="str">
+        <v>Discount, Percentages, Sale</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>Castle Defender</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Factors, Multiples &amp; Primes</v>
+      </c>
+      <c r="C21" t="str">
+        <v>What is the Greatest Common Divisor (GCD) of 36 and 54 to reinforce the fortress gate?</v>
+      </c>
+      <c r="D21" t="str">
+        <v>9</v>
+      </c>
+      <c r="E21" t="str">
+        <v>12</v>
+      </c>
+      <c r="F21" t="str">
+        <v>18</v>
+      </c>
+      <c r="G21" t="str">
+        <v>27</v>
+      </c>
+      <c r="H21" t="str">
+        <v>C</v>
+      </c>
+      <c r="I21" t="str">
+        <v>Factors of 36: 1, 2, 3, 4, 6, 9, 12, 18, 36. Factors of 54: 1, 2, 3, 6, 9, 18, 27, 54. GCD = 18.</v>
+      </c>
+      <c r="J21" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="K21" t="str">
+        <v>GCD, Factors, Castle</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>Castle Defender</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Factors, Multiples &amp; Primes</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Which of the following numbers is prime?</v>
+      </c>
+      <c r="D22" t="str">
+        <v>51</v>
+      </c>
+      <c r="E22" t="str">
+        <v>57</v>
+      </c>
+      <c r="F22" t="str">
+        <v>61</v>
+      </c>
+      <c r="G22" t="str">
+        <v>63</v>
+      </c>
+      <c r="H22" t="str">
+        <v>C</v>
+      </c>
+      <c r="I22" t="str">
+        <v>61 has only 1 and 61 as factors. (51 = 3×17, 57 = 3×19, 63 = 3×21).</v>
+      </c>
+      <c r="J22" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="K22" t="str">
+        <v>Prime Numbers, Factors</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>Space Station Alpha</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Angles &amp; Triangles</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Two angles of a navigation triangle measure 65° and 45°. What is the third angle?</v>
+      </c>
+      <c r="D23" t="str">
+        <v>60°</v>
+      </c>
+      <c r="E23" t="str">
+        <v>70°</v>
+      </c>
+      <c r="F23" t="str">
+        <v>80°</v>
+      </c>
+      <c r="G23" t="str">
+        <v>90°</v>
+      </c>
+      <c r="H23" t="str">
+        <v>B</v>
+      </c>
+      <c r="I23" t="str">
+        <v>Sum of angles in a triangle = 180°. Third angle = 180° - 110° = 70°.</v>
+      </c>
+      <c r="J23" t="str">
+        <v>Easy</v>
+      </c>
+      <c r="K23" t="str">
+        <v>Triangles, Angles, Space Station</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>Space Station Alpha</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Angles &amp; Triangles</v>
+      </c>
+      <c r="C24" t="str">
+        <v>What type of angle measures exactly 135°?</v>
+      </c>
+      <c r="D24" t="str">
+        <v>Acute angle</v>
+      </c>
+      <c r="E24" t="str">
+        <v>Right angle</v>
+      </c>
+      <c r="F24" t="str">
+        <v>Obtuse angle</v>
+      </c>
+      <c r="G24" t="str">
+        <v>Reflex angle</v>
+      </c>
+      <c r="H24" t="str">
+        <v>C</v>
+      </c>
+      <c r="I24" t="str">
+        <v>An angle between 90° and 180° is an obtuse angle.</v>
+      </c>
+      <c r="J24" t="str">
+        <v>Easy</v>
+      </c>
+      <c r="K24" t="str">
+        <v>Angle Classification, Geometry</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>Market Tycoon</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Money, Profit &amp; Loss</v>
+      </c>
+      <c r="C25" t="str">
+        <v>A shopkeeper buys a trading card for  and sells it for . What is the profit made?</v>
+      </c>
+      <c r="D25" t="str">
+        <v/>
+      </c>
+      <c r="E25" t="str">
+        <v/>
+      </c>
+      <c r="F25" t="str">
+        <v/>
+      </c>
+      <c r="G25" t="str">
+        <v/>
+      </c>
+      <c r="H25" t="str">
+        <v>B</v>
+      </c>
+      <c r="I25" t="str">
+        <v>Profit = Selling Price - Cost Price =  -  = .</v>
+      </c>
+      <c r="J25" t="str">
+        <v>Easy</v>
+      </c>
+      <c r="K25" t="str">
+        <v>Profit and Loss, Money, Trading</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>Market Tycoon</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Money, Profit &amp; Loss</v>
+      </c>
+      <c r="C26" t="str">
+        <v>If 6 arcade game tokens cost .00, what is the cost of 10 tokens?</v>
+      </c>
+      <c r="D26" t="str">
+        <v>.50</v>
+      </c>
+      <c r="E26" t="str">
+        <v>.00</v>
+      </c>
+      <c r="F26" t="str">
+        <v>.00</v>
+      </c>
+      <c r="G26" t="str">
+        <v>.00</v>
+      </c>
+      <c r="H26" t="str">
+        <v>B</v>
+      </c>
+      <c r="I26" t="str">
+        <v>Cost per token = .00 ÷ 6 = .50. Cost for 10 = .50 × 10 = .00.</v>
+      </c>
+      <c r="J26" t="str">
+        <v>Easy</v>
+      </c>
+      <c r="K26" t="str">
+        <v>Unit Price, Proportions, Money</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>Park Planner</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Position &amp; Transformation</v>
+      </c>
+      <c r="C27" t="str">
+        <v>When the fountain coordinate (4, -3) is translated 3 units left and 5 units up, what is its new location?</v>
+      </c>
+      <c r="D27" t="str">
+        <v>(1, 2)</v>
+      </c>
+      <c r="E27" t="str">
+        <v>(7, 2)</v>
+      </c>
+      <c r="F27" t="str">
+        <v>(1, -8)</v>
+      </c>
+      <c r="G27" t="str">
+        <v>(7, -8)</v>
+      </c>
+      <c r="H27" t="str">
+        <v>A</v>
+      </c>
+      <c r="I27" t="str">
+        <v>New x = 4 - 3 = 1. New y = -3 + 5 = 2. New position = (1, 2).</v>
+      </c>
+      <c r="J27" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="K27" t="str">
+        <v>Transformations, Translation, Grid</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>Park Planner</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Position &amp; Transformation</v>
+      </c>
+      <c r="C28" t="str">
+        <v>In which quadrant does the park bench coordinate (-5, 6) lie?</v>
+      </c>
+      <c r="D28" t="str">
+        <v>Quadrant I</v>
+      </c>
+      <c r="E28" t="str">
+        <v>Quadrant II</v>
+      </c>
+      <c r="F28" t="str">
+        <v>Quadrant III</v>
+      </c>
+      <c r="G28" t="str">
+        <v>Quadrant IV</v>
+      </c>
+      <c r="H28" t="str">
+        <v>B</v>
+      </c>
+      <c r="I28" t="str">
+        <v>Negative x and positive y is located in Quadrant II.</v>
+      </c>
+      <c r="J28" t="str">
+        <v>Easy</v>
+      </c>
+      <c r="K28" t="str">
+        <v>Cartesian Plane, Quadrants, Coordinates</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>GraphWorks</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Data Handling &amp; Graphs</v>
+      </c>
+      <c r="C29" t="str">
+        <v>Find the median of this dataset of student high scores: 12, 15, 18, 22, 29, 31, 35</v>
+      </c>
+      <c r="D29" t="str">
+        <v>18</v>
+      </c>
+      <c r="E29" t="str">
+        <v>20</v>
+      </c>
+      <c r="F29" t="str">
+        <v>22</v>
+      </c>
+      <c r="G29" t="str">
+        <v>29</v>
+      </c>
+      <c r="H29" t="str">
+        <v>C</v>
+      </c>
+      <c r="I29" t="str">
+        <v>The numbers are in order; the middle value (4th of 7 items) is 22.</v>
+      </c>
+      <c r="J29" t="str">
+        <v>Easy</v>
+      </c>
+      <c r="K29" t="str">
+        <v>Statistics, Median, Graphs</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>GraphWorks</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Data Handling &amp; Graphs</v>
+      </c>
+      <c r="C30" t="str">
+        <v>A bar chart shows daily arcade visits: Mon (40), Tue (50), Wed (60), Thu (70), Fri (80). What is the mean daily visit count?</v>
+      </c>
+      <c r="D30" t="str">
+        <v>55 visits</v>
+      </c>
+      <c r="E30" t="str">
+        <v>60 visits</v>
+      </c>
+      <c r="F30" t="str">
+        <v>65 visits</v>
+      </c>
+      <c r="G30" t="str">
+        <v>70 visits</v>
+      </c>
+      <c r="H30" t="str">
+        <v>B</v>
+      </c>
+      <c r="I30" t="str">
+        <v>Mean = (40 + 50 + 60 + 70 + 80) ÷ 5 = 300 ÷ 5 = 60 visits.</v>
+      </c>
+      <c r="J30" t="str">
+        <v>Easy</v>
+      </c>
+      <c r="K30" t="str">
+        <v>Mean, Data Handling, Bar Chart</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K16"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K30"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -998,7 +1392,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Follow these simple 8 steps to import custom questions for your students.</v>
+        <v>Follow these simple steps to import custom questions for your students.</v>
       </c>
     </row>
     <row r="4">
@@ -1020,7 +1414,7 @@
         <v>Choose the Activity</v>
       </c>
       <c r="C5" t="str">
-        <v>Select from the 13 official arcade games (e.g. "GraphWorks" or "The Chocolate Factory").</v>
+        <v>Select from the 13 official arcade games.</v>
       </c>
     </row>
     <row r="6">
@@ -1031,7 +1425,7 @@
         <v>Verify the Math Topic</v>
       </c>
       <c r="C6" t="str">
-        <v>The topic must match the activity's curriculum subject (refer to the "Activity List" sheet).</v>
+        <v>The topic must match the activity's curriculum subject.</v>
       </c>
     </row>
     <row r="7">
@@ -1042,7 +1436,7 @@
         <v>Enter Your Question</v>
       </c>
       <c r="C7" t="str">
-        <v>Write the complete question prompt. Mathematical symbols (+, -, ×, ÷, ², √, etc.) are fully supported.</v>
+        <v>Write the complete question prompt.</v>
       </c>
     </row>
     <row r="8">
@@ -1053,7 +1447,7 @@
         <v>Enter Four Options</v>
       </c>
       <c r="C8" t="str">
-        <v>You must provide all 4 distinct answer choices: Option A, Option B, Option C, and Option D.</v>
+        <v>You must provide all 4 distinct answer choices.</v>
       </c>
     </row>
     <row r="9">
@@ -1064,7 +1458,7 @@
         <v>Select Correct Answer</v>
       </c>
       <c r="C9" t="str">
-        <v>Enter "A", "B", "C", or "D" under the Correct Answer column.</v>
+        <v>Enter A, B, C, or D.</v>
       </c>
     </row>
     <row r="10">
@@ -1075,7 +1469,7 @@
         <v>Add Feedback &amp; Difficulty</v>
       </c>
       <c r="C10" t="str">
-        <v>Optionally add an explanation (displayed as learning feedback) and set Difficulty to Easy, Medium, or Hard.</v>
+        <v>Optionally add an explanation and difficulty.</v>
       </c>
     </row>
     <row r="11">
@@ -1097,7 +1491,7 @@
         <v>Upload into Arcade</v>
       </c>
       <c r="C12" t="str">
-        <v>Open the Question Manager in Skillizee Arcade, click "Import Excel", preview verified questions, and click Import!</v>
+        <v>Open Question Manager, click Import Excel, verify, and import.</v>
       </c>
     </row>
   </sheetData>
@@ -1109,246 +1503,13 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K6"/>
-  <cols>
-    <col min="1" max="1" width="26.83203125" customWidth="1"/>
-    <col min="2" max="2" width="28.83203125" customWidth="1"/>
-    <col min="3" max="3" width="60.83203125" customWidth="1"/>
-    <col min="4" max="4" width="20.83203125" customWidth="1"/>
-    <col min="5" max="5" width="20.83203125" customWidth="1"/>
-    <col min="6" max="6" width="20.83203125" customWidth="1"/>
-    <col min="7" max="7" width="20.83203125" customWidth="1"/>
-    <col min="8" max="8" width="16.83203125" customWidth="1"/>
-    <col min="9" max="9" width="45.83203125" customWidth="1"/>
-    <col min="10" max="10" width="14.83203125" customWidth="1"/>
-    <col min="11" max="11" width="30.83203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Activity</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Topic</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Question</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Option A</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Option B</v>
-      </c>
-      <c r="F1" t="str">
-        <v>Option C</v>
-      </c>
-      <c r="G1" t="str">
-        <v>Option D</v>
-      </c>
-      <c r="H1" t="str">
-        <v>Correct Answer</v>
-      </c>
-      <c r="I1" t="str">
-        <v>Explanation</v>
-      </c>
-      <c r="J1" t="str">
-        <v>Difficulty</v>
-      </c>
-      <c r="K1" t="str">
-        <v>Tags</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Graphworks</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Data Handling &amp; Graphs</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Which ordered pair represents 3 units right on the x-axis and 4 units up on the y-axis?</v>
-      </c>
-      <c r="D2" t="str">
-        <v>(4, 3)</v>
-      </c>
-      <c r="E2" t="str">
-        <v>(3, 4)</v>
-      </c>
-      <c r="F2" t="str">
-        <v>(3, 0)</v>
-      </c>
-      <c r="G2" t="str">
-        <v>(0, 4)</v>
-      </c>
-      <c r="H2" t="str">
-        <v>B</v>
-      </c>
-      <c r="I2" t="str">
-        <v>Coordinates are written as (x, y). Moving 3 units right gives x = 3, and 4 units up gives y = 4, resulting in (3, 4).</v>
-      </c>
-      <c r="J2" t="str">
-        <v>Easy</v>
-      </c>
-      <c r="K2" t="str">
-        <v>Coordinates, Grid, Plotting</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>The Chocolate Factory</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Fractions</v>
-      </c>
-      <c r="C3" t="str">
-        <v>A chocolate batch uses 3/4 cup of melted cocoa. How much cocoa is needed for 3 full batches?</v>
-      </c>
-      <c r="D3" t="str">
-        <v>2 1/4 cups</v>
-      </c>
-      <c r="E3" t="str">
-        <v>1 1/2 cups</v>
-      </c>
-      <c r="F3" t="str">
-        <v>3 cups</v>
-      </c>
-      <c r="G3" t="str">
-        <v>9/4 cups</v>
-      </c>
-      <c r="H3" t="str">
-        <v>A</v>
-      </c>
-      <c r="I3" t="str">
-        <v>3 × 3/4 = 9/4 = 2 1/4 cups of cocoa.</v>
-      </c>
-      <c r="J3" t="str">
-        <v>Medium</v>
-      </c>
-      <c r="K3" t="str">
-        <v>Fractions, Multiplication, Mixed Numbers</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>Percentage Harvest</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Percentages</v>
-      </c>
-      <c r="C4" t="str">
-        <v>What is 20% of 80 kg of harvest apples?</v>
-      </c>
-      <c r="D4" t="str">
-        <v>12 kg</v>
-      </c>
-      <c r="E4" t="str">
-        <v>16 kg</v>
-      </c>
-      <c r="F4" t="str">
-        <v>18 kg</v>
-      </c>
-      <c r="G4" t="str">
-        <v>20 kg</v>
-      </c>
-      <c r="H4" t="str">
-        <v>B</v>
-      </c>
-      <c r="I4" t="str">
-        <v>20% of 80 = 0.2 × 80 = 16 kg.</v>
-      </c>
-      <c r="J4" t="str">
-        <v>Easy</v>
-      </c>
-      <c r="K4" t="str">
-        <v>Percentages, Harvest, Calculations</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>Park Planner</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Position &amp; Transformation</v>
-      </c>
-      <c r="C5" t="str">
-        <v>When the point (2, 5) is reflected over the y-axis, what are its new coordinates?</v>
-      </c>
-      <c r="D5" t="str">
-        <v>(-2, 5)</v>
-      </c>
-      <c r="E5" t="str">
-        <v>(2, -5)</v>
-      </c>
-      <c r="F5" t="str">
-        <v>(-2, -5)</v>
-      </c>
-      <c r="G5" t="str">
-        <v>(5, 2)</v>
-      </c>
-      <c r="H5" t="str">
-        <v>A</v>
-      </c>
-      <c r="I5" t="str">
-        <v>Reflecting over the y-axis negates the x-coordinate while y remains unchanged: (-2, 5).</v>
-      </c>
-      <c r="J5" t="str">
-        <v>Medium</v>
-      </c>
-      <c r="K5" t="str">
-        <v>Transformations, Reflection, Coordinates</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>Ratio Rush</v>
-      </c>
-      <c r="B6" t="str">
-        <v>Ratios, Rates &amp; Proportions</v>
-      </c>
-      <c r="C6" t="str">
-        <v>A film studio uses 2 cameras for every 3 actors. If there are 12 actors, how many cameras are needed?</v>
-      </c>
-      <c r="D6" t="str">
-        <v>6</v>
-      </c>
-      <c r="E6" t="str">
-        <v>8</v>
-      </c>
-      <c r="F6" t="str">
-        <v>9</v>
-      </c>
-      <c r="G6" t="str">
-        <v>10</v>
-      </c>
-      <c r="H6" t="str">
-        <v>B</v>
-      </c>
-      <c r="I6" t="str">
-        <v>Scale factor is 12 ÷ 3 = 4. Cameras = 2 × 4 = 8.</v>
-      </c>
-      <c r="J6" t="str">
-        <v>Easy</v>
-      </c>
-      <c r="K6" t="str">
-        <v>Ratio, Scaling, Unit Rate</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K6"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:E14"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
-    <col min="3" max="3" width="35.83203125" customWidth="1"/>
-    <col min="4" max="4" width="40.83203125" customWidth="1"/>
+    <col min="3" max="3" width="32.83203125" customWidth="1"/>
+    <col min="4" max="4" width="36.83203125" customWidth="1"/>
+    <col min="5" max="5" width="22.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1364,6 +1525,9 @@
       <c r="D1" t="str">
         <v>Dropdown Value</v>
       </c>
+      <c r="E1" t="str">
+        <v>Activity ID</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -1376,7 +1540,10 @@
         <v>Place Value &amp; Decimals</v>
       </c>
       <c r="D2" t="str">
-        <v>Math Escape Vault — Place Value &amp; Decimals</v>
+        <v>Math Escape Vault — Decimals</v>
+      </c>
+      <c r="E2" t="str">
+        <v>math-escape-vault</v>
       </c>
     </row>
     <row r="3">
@@ -1384,13 +1551,16 @@
         <v>Cab #02</v>
       </c>
       <c r="B3" t="str">
-        <v>The Great Number Railway</v>
+        <v>The Chocolate Factory</v>
       </c>
       <c r="C3" t="str">
-        <v>Operations &amp; Rounding</v>
+        <v>Fractions</v>
       </c>
       <c r="D3" t="str">
-        <v>The Great Number Railway — Operations &amp; Rounding</v>
+        <v>The Chocolate Factory — Fractions</v>
+      </c>
+      <c r="E3" t="str">
+        <v>the-chocolate-factory</v>
       </c>
     </row>
     <row r="4">
@@ -1398,13 +1568,16 @@
         <v>Cab #03</v>
       </c>
       <c r="B4" t="str">
-        <v>Carnival of Chance</v>
+        <v>Ratio Rush</v>
       </c>
       <c r="C4" t="str">
-        <v>Probability</v>
+        <v>Ratios, Rates &amp; Proportions</v>
       </c>
       <c r="D4" t="str">
-        <v>Carnival of Chance — Probability</v>
+        <v>Ratio Rush — Ratios &amp; Proportions</v>
+      </c>
+      <c r="E4" t="str">
+        <v>ratio-rush</v>
       </c>
     </row>
     <row r="5">
@@ -1412,13 +1585,16 @@
         <v>Cab #04</v>
       </c>
       <c r="B5" t="str">
-        <v>Blueprint Blitz</v>
+        <v>Shape Shifter Arena</v>
       </c>
       <c r="C5" t="str">
-        <v>Shapes, Area &amp; Volume</v>
+        <v>Geometry &amp; Symmetry</v>
       </c>
       <c r="D5" t="str">
-        <v>Blueprint Blitz — Shapes, Area &amp; Volume</v>
+        <v>Shape Shifter Arena — Geometry &amp; Symmetry</v>
+      </c>
+      <c r="E5" t="str">
+        <v>shape-shifter-arena</v>
       </c>
     </row>
     <row r="6">
@@ -1426,13 +1602,16 @@
         <v>Cab #05</v>
       </c>
       <c r="B6" t="str">
-        <v>Equation Mission Control</v>
+        <v>Time Warp Train</v>
       </c>
       <c r="C6" t="str">
-        <v>Expressions &amp; Equations</v>
+        <v>Time &amp; Measurement</v>
       </c>
       <c r="D6" t="str">
-        <v>Equation Mission Control — Expressions &amp; Equations</v>
+        <v>Time Warp Train — Time &amp; Measurement</v>
+      </c>
+      <c r="E6" t="str">
+        <v>time-warp-train</v>
       </c>
     </row>
     <row r="7">
@@ -1440,13 +1619,16 @@
         <v>Cab #06</v>
       </c>
       <c r="B7" t="str">
-        <v>Pattern Racers</v>
+        <v>Formula 1 Speedway</v>
       </c>
       <c r="C7" t="str">
-        <v>Sequences &amp; Functions</v>
+        <v>Algebra &amp; Sequences</v>
       </c>
       <c r="D7" t="str">
-        <v>Pattern Racers — Sequences &amp; Functions</v>
+        <v>Formula 1 Speedway — Algebra &amp; Sequences</v>
+      </c>
+      <c r="E7" t="str">
+        <v>formula-1-speedway</v>
       </c>
     </row>
     <row r="8">
@@ -1454,13 +1636,16 @@
         <v>Cab #07</v>
       </c>
       <c r="B8" t="str">
-        <v>Decimal Delivery Network</v>
+        <v>Deep Sea Diver</v>
       </c>
       <c r="C8" t="str">
-        <v>Decimals</v>
+        <v>Integers &amp; Negative Numbers</v>
       </c>
       <c r="D8" t="str">
-        <v>Decimal Delivery Network — Decimals</v>
+        <v>Deep Sea Diver — Negative Numbers</v>
+      </c>
+      <c r="E8" t="str">
+        <v>deep-sea-diver</v>
       </c>
     </row>
     <row r="9">
@@ -1468,13 +1653,16 @@
         <v>Cab #08</v>
       </c>
       <c r="B9" t="str">
-        <v>The Solar Forge</v>
+        <v>Percentage Harvest</v>
       </c>
       <c r="C9" t="str">
-        <v>Angles, Protractor &amp; Constructions</v>
+        <v>Percentages</v>
       </c>
       <c r="D9" t="str">
-        <v>The Solar Forge — Angles, Protractor &amp; Constructions</v>
+        <v>Percentage Harvest — Percentages</v>
+      </c>
+      <c r="E9" t="str">
+        <v>percentage-harvest</v>
       </c>
     </row>
     <row r="10">
@@ -1482,13 +1670,16 @@
         <v>Cab #09</v>
       </c>
       <c r="B10" t="str">
-        <v>The Chocolate Factory</v>
+        <v>Castle Defender</v>
       </c>
       <c r="C10" t="str">
-        <v>Fractions</v>
+        <v>Factors, Multiples &amp; Primes</v>
       </c>
       <c r="D10" t="str">
-        <v>The Chocolate Factory — Fractions</v>
+        <v>Castle Defender — Factors &amp; Primes</v>
+      </c>
+      <c r="E10" t="str">
+        <v>castle-defender</v>
       </c>
     </row>
     <row r="11">
@@ -1496,13 +1687,16 @@
         <v>Cab #10</v>
       </c>
       <c r="B11" t="str">
-        <v>Graphworks</v>
+        <v>Space Station Alpha</v>
       </c>
       <c r="C11" t="str">
-        <v>Data Handling &amp; Graphs</v>
+        <v>Angles &amp; Triangles</v>
       </c>
       <c r="D11" t="str">
-        <v>Graphworks — Data Handling &amp; Graphs</v>
+        <v>Space Station Alpha — Angles &amp; Triangles</v>
+      </c>
+      <c r="E11" t="str">
+        <v>space-station-alpha</v>
       </c>
     </row>
     <row r="12">
@@ -1510,13 +1704,16 @@
         <v>Cab #11</v>
       </c>
       <c r="B12" t="str">
-        <v>Percentage Harvest</v>
+        <v>Market Tycoon</v>
       </c>
       <c r="C12" t="str">
-        <v>Percentages</v>
+        <v>Money, Profit &amp; Loss</v>
       </c>
       <c r="D12" t="str">
-        <v>Percentage Harvest — Percentages</v>
+        <v>Market Tycoon — Profit &amp; Loss</v>
+      </c>
+      <c r="E12" t="str">
+        <v>market-tycoon</v>
       </c>
     </row>
     <row r="13">
@@ -1530,7 +1727,10 @@
         <v>Position &amp; Transformation</v>
       </c>
       <c r="D13" t="str">
-        <v>Park Planner — Position &amp; Transformation</v>
+        <v>Park Planner — Transformation</v>
+      </c>
+      <c r="E13" t="str">
+        <v>park-planner</v>
       </c>
     </row>
     <row r="14">
@@ -1538,18 +1738,21 @@
         <v>Cab #13</v>
       </c>
       <c r="B14" t="str">
-        <v>Ratio Rush</v>
+        <v>GraphWorks</v>
       </c>
       <c r="C14" t="str">
-        <v>Ratios, Rates &amp; Proportions</v>
+        <v>Data Handling &amp; Graphs</v>
       </c>
       <c r="D14" t="str">
-        <v>Ratio Rush — Ratios, Rates &amp; Proportions</v>
+        <v>GraphWorks — Graphs &amp; Charts</v>
+      </c>
+      <c r="E14" t="str">
+        <v>graphworks</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E14"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>